<commit_message>
Correções + processo mecanizou e compel
</commit_message>
<xml_diff>
--- a/planilhas/Planilha de Base para Cotacao.xlsx
+++ b/planilhas/Planilha de Base para Cotacao.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a19316afdd125d6/Documentos/GitHub/hawks-automations/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23C3C222-9546-4B10-82B8-A65D6D2EFB03}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A4F1FFD-D5BE-4EBF-9D34-ACCAE02760C1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{AB0A4C4E-1938-46F3-8FAE-9EC8B05F0B3E}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -78,11 +78,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Var(--font-family-montserrat)"/>
     </font>
     <font>
       <sz val="10"/>
@@ -110,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -119,9 +114,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -478,78 +470,81 @@
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="5"/>
-      <c r="C2" s="4"/>
+      <c r="A2" s="4"/>
+      <c r="G2" s="1" t="e">
+        <f>MEDIAN(C2,D2,E2,F2)*1.8</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="5"/>
+      <c r="A3" s="4"/>
       <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="5"/>
+      <c r="A4" s="4"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="5"/>
+      <c r="A5" s="4"/>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="5"/>
+      <c r="A6" s="4"/>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="5"/>
+      <c r="A7" s="4"/>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="5"/>
+      <c r="A8" s="4"/>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="5"/>
+      <c r="A9" s="4"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="5"/>
+      <c r="A10" s="4"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="5"/>
+      <c r="A11" s="4"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="5"/>
+      <c r="A12" s="4"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="5"/>
+      <c r="A13" s="4"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="5"/>
+      <c r="A14" s="4"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="5"/>
+      <c r="A15" s="4"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="5"/>
+      <c r="A16" s="4"/>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="5"/>
+      <c r="A17" s="4"/>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="5"/>
+      <c r="A18" s="4"/>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="5"/>
+      <c r="A19" s="4"/>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="5"/>
+      <c r="A20" s="4"/>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" s="5"/>
+      <c r="A21" s="4"/>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" s="5"/>
+      <c r="A22" s="4"/>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" s="5"/>
+      <c r="A23" s="4"/>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="5"/>
+      <c r="A24" s="4"/>
     </row>
     <row r="25" spans="1:1">
-      <c r="A25" s="5"/>
+      <c r="A25" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
Refatoração e início do segundo processo.
Refatoração: adição de verificações em caso de indisponibilidade da peça.
</commit_message>
<xml_diff>
--- a/planilhas/Planilha de Base para Cotacao.xlsx
+++ b/planilhas/Planilha de Base para Cotacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a19316afdd125d6/Documentos/GitHub/hawks-automations/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="102" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6312C9EA-B1ED-4883-9FA8-8ABCD49C1767}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3DA2ADD-C9EA-4CC3-8D51-49BBE95BCFBA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{AB0A4C4E-1938-46F3-8FAE-9EC8B05F0B3E}"/>
   </bookViews>
@@ -137,9 +137,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -177,7 +177,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -283,7 +283,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -425,7 +425,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -438,10 +438,9 @@
   <cols>
     <col min="1" max="1" width="17.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="1"/>
+    <col min="5" max="6" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -1772,6 +1771,137 @@
     </row>
   </sheetData>
   <mergeCells count="144">
+    <mergeCell ref="A431:A433"/>
+    <mergeCell ref="A416:A418"/>
+    <mergeCell ref="A419:A421"/>
+    <mergeCell ref="A422:A424"/>
+    <mergeCell ref="A425:A427"/>
+    <mergeCell ref="A428:A430"/>
+    <mergeCell ref="A401:A403"/>
+    <mergeCell ref="A404:A406"/>
+    <mergeCell ref="A407:A409"/>
+    <mergeCell ref="A410:A412"/>
+    <mergeCell ref="A413:A415"/>
+    <mergeCell ref="A386:A388"/>
+    <mergeCell ref="A389:A391"/>
+    <mergeCell ref="A392:A394"/>
+    <mergeCell ref="A395:A397"/>
+    <mergeCell ref="A398:A400"/>
+    <mergeCell ref="A371:A373"/>
+    <mergeCell ref="A374:A376"/>
+    <mergeCell ref="A377:A379"/>
+    <mergeCell ref="A380:A382"/>
+    <mergeCell ref="A383:A385"/>
+    <mergeCell ref="A356:A358"/>
+    <mergeCell ref="A359:A361"/>
+    <mergeCell ref="A362:A364"/>
+    <mergeCell ref="A365:A367"/>
+    <mergeCell ref="A368:A370"/>
+    <mergeCell ref="A341:A343"/>
+    <mergeCell ref="A344:A346"/>
+    <mergeCell ref="A347:A349"/>
+    <mergeCell ref="A350:A352"/>
+    <mergeCell ref="A353:A355"/>
+    <mergeCell ref="A326:A328"/>
+    <mergeCell ref="A329:A331"/>
+    <mergeCell ref="A332:A334"/>
+    <mergeCell ref="A335:A337"/>
+    <mergeCell ref="A338:A340"/>
+    <mergeCell ref="A311:A313"/>
+    <mergeCell ref="A314:A316"/>
+    <mergeCell ref="A317:A319"/>
+    <mergeCell ref="A320:A322"/>
+    <mergeCell ref="A323:A325"/>
+    <mergeCell ref="A296:A298"/>
+    <mergeCell ref="A299:A301"/>
+    <mergeCell ref="A302:A304"/>
+    <mergeCell ref="A305:A307"/>
+    <mergeCell ref="A308:A310"/>
+    <mergeCell ref="A281:A283"/>
+    <mergeCell ref="A284:A286"/>
+    <mergeCell ref="A287:A289"/>
+    <mergeCell ref="A290:A292"/>
+    <mergeCell ref="A293:A295"/>
+    <mergeCell ref="A266:A268"/>
+    <mergeCell ref="A269:A271"/>
+    <mergeCell ref="A272:A274"/>
+    <mergeCell ref="A275:A277"/>
+    <mergeCell ref="A278:A280"/>
+    <mergeCell ref="A251:A253"/>
+    <mergeCell ref="A254:A256"/>
+    <mergeCell ref="A257:A259"/>
+    <mergeCell ref="A260:A262"/>
+    <mergeCell ref="A263:A265"/>
+    <mergeCell ref="A236:A238"/>
+    <mergeCell ref="A239:A241"/>
+    <mergeCell ref="A242:A244"/>
+    <mergeCell ref="A245:A247"/>
+    <mergeCell ref="A248:A250"/>
+    <mergeCell ref="A221:A223"/>
+    <mergeCell ref="A224:A226"/>
+    <mergeCell ref="A227:A229"/>
+    <mergeCell ref="A230:A232"/>
+    <mergeCell ref="A233:A235"/>
+    <mergeCell ref="A206:A208"/>
+    <mergeCell ref="A209:A211"/>
+    <mergeCell ref="A212:A214"/>
+    <mergeCell ref="A215:A217"/>
+    <mergeCell ref="A218:A220"/>
+    <mergeCell ref="A191:A193"/>
+    <mergeCell ref="A194:A196"/>
+    <mergeCell ref="A197:A199"/>
+    <mergeCell ref="A200:A202"/>
+    <mergeCell ref="A203:A205"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A181"/>
+    <mergeCell ref="A182:A184"/>
+    <mergeCell ref="A185:A187"/>
+    <mergeCell ref="A188:A190"/>
+    <mergeCell ref="A161:A163"/>
+    <mergeCell ref="A164:A166"/>
+    <mergeCell ref="A167:A169"/>
+    <mergeCell ref="A170:A172"/>
+    <mergeCell ref="A173:A175"/>
+    <mergeCell ref="A146:A148"/>
+    <mergeCell ref="A149:A151"/>
+    <mergeCell ref="A152:A154"/>
+    <mergeCell ref="A155:A157"/>
+    <mergeCell ref="A158:A160"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="A134:A136"/>
+    <mergeCell ref="A137:A139"/>
+    <mergeCell ref="A140:A142"/>
+    <mergeCell ref="A143:A145"/>
+    <mergeCell ref="A116:A118"/>
+    <mergeCell ref="A119:A121"/>
+    <mergeCell ref="A122:A124"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="A113:A115"/>
+    <mergeCell ref="A86:A88"/>
+    <mergeCell ref="A89:A91"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="A98:A100"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A74:A76"/>
+    <mergeCell ref="A77:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A56:A58"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="A68:A70"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="A53:A55"/>
     <mergeCell ref="A26:A28"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="A32:A34"/>
@@ -1785,137 +1915,6 @@
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A56:A58"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="A68:A70"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="A53:A55"/>
-    <mergeCell ref="A86:A88"/>
-    <mergeCell ref="A89:A91"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A98:A100"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A116:A118"/>
-    <mergeCell ref="A119:A121"/>
-    <mergeCell ref="A122:A124"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A112"/>
-    <mergeCell ref="A113:A115"/>
-    <mergeCell ref="A146:A148"/>
-    <mergeCell ref="A149:A151"/>
-    <mergeCell ref="A152:A154"/>
-    <mergeCell ref="A155:A157"/>
-    <mergeCell ref="A158:A160"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="A134:A136"/>
-    <mergeCell ref="A137:A139"/>
-    <mergeCell ref="A140:A142"/>
-    <mergeCell ref="A143:A145"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A181"/>
-    <mergeCell ref="A182:A184"/>
-    <mergeCell ref="A185:A187"/>
-    <mergeCell ref="A188:A190"/>
-    <mergeCell ref="A161:A163"/>
-    <mergeCell ref="A164:A166"/>
-    <mergeCell ref="A167:A169"/>
-    <mergeCell ref="A170:A172"/>
-    <mergeCell ref="A173:A175"/>
-    <mergeCell ref="A206:A208"/>
-    <mergeCell ref="A209:A211"/>
-    <mergeCell ref="A212:A214"/>
-    <mergeCell ref="A215:A217"/>
-    <mergeCell ref="A218:A220"/>
-    <mergeCell ref="A191:A193"/>
-    <mergeCell ref="A194:A196"/>
-    <mergeCell ref="A197:A199"/>
-    <mergeCell ref="A200:A202"/>
-    <mergeCell ref="A203:A205"/>
-    <mergeCell ref="A236:A238"/>
-    <mergeCell ref="A239:A241"/>
-    <mergeCell ref="A242:A244"/>
-    <mergeCell ref="A245:A247"/>
-    <mergeCell ref="A248:A250"/>
-    <mergeCell ref="A221:A223"/>
-    <mergeCell ref="A224:A226"/>
-    <mergeCell ref="A227:A229"/>
-    <mergeCell ref="A230:A232"/>
-    <mergeCell ref="A233:A235"/>
-    <mergeCell ref="A266:A268"/>
-    <mergeCell ref="A269:A271"/>
-    <mergeCell ref="A272:A274"/>
-    <mergeCell ref="A275:A277"/>
-    <mergeCell ref="A278:A280"/>
-    <mergeCell ref="A251:A253"/>
-    <mergeCell ref="A254:A256"/>
-    <mergeCell ref="A257:A259"/>
-    <mergeCell ref="A260:A262"/>
-    <mergeCell ref="A263:A265"/>
-    <mergeCell ref="A296:A298"/>
-    <mergeCell ref="A299:A301"/>
-    <mergeCell ref="A302:A304"/>
-    <mergeCell ref="A305:A307"/>
-    <mergeCell ref="A308:A310"/>
-    <mergeCell ref="A281:A283"/>
-    <mergeCell ref="A284:A286"/>
-    <mergeCell ref="A287:A289"/>
-    <mergeCell ref="A290:A292"/>
-    <mergeCell ref="A293:A295"/>
-    <mergeCell ref="A326:A328"/>
-    <mergeCell ref="A329:A331"/>
-    <mergeCell ref="A332:A334"/>
-    <mergeCell ref="A335:A337"/>
-    <mergeCell ref="A338:A340"/>
-    <mergeCell ref="A311:A313"/>
-    <mergeCell ref="A314:A316"/>
-    <mergeCell ref="A317:A319"/>
-    <mergeCell ref="A320:A322"/>
-    <mergeCell ref="A323:A325"/>
-    <mergeCell ref="A356:A358"/>
-    <mergeCell ref="A359:A361"/>
-    <mergeCell ref="A362:A364"/>
-    <mergeCell ref="A365:A367"/>
-    <mergeCell ref="A368:A370"/>
-    <mergeCell ref="A341:A343"/>
-    <mergeCell ref="A344:A346"/>
-    <mergeCell ref="A347:A349"/>
-    <mergeCell ref="A350:A352"/>
-    <mergeCell ref="A353:A355"/>
-    <mergeCell ref="A386:A388"/>
-    <mergeCell ref="A389:A391"/>
-    <mergeCell ref="A392:A394"/>
-    <mergeCell ref="A395:A397"/>
-    <mergeCell ref="A398:A400"/>
-    <mergeCell ref="A371:A373"/>
-    <mergeCell ref="A374:A376"/>
-    <mergeCell ref="A377:A379"/>
-    <mergeCell ref="A380:A382"/>
-    <mergeCell ref="A383:A385"/>
-    <mergeCell ref="A431:A433"/>
-    <mergeCell ref="A416:A418"/>
-    <mergeCell ref="A419:A421"/>
-    <mergeCell ref="A422:A424"/>
-    <mergeCell ref="A425:A427"/>
-    <mergeCell ref="A428:A430"/>
-    <mergeCell ref="A401:A403"/>
-    <mergeCell ref="A404:A406"/>
-    <mergeCell ref="A407:A409"/>
-    <mergeCell ref="A410:A412"/>
-    <mergeCell ref="A413:A415"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Segunda rodada do processo do kdapeca pronta
</commit_message>
<xml_diff>
--- a/planilhas/Planilha de Base para Cotacao.xlsx
+++ b/planilhas/Planilha de Base para Cotacao.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a19316afdd125d6/Documentos/GitHub/hawks-automations/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="120" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3DA2ADD-C9EA-4CC3-8D51-49BBE95BCFBA}"/>
+  <xr:revisionPtr revIDLastSave="276" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA88737E-75B2-4ED2-AA61-A48FA5D38C95}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{AB0A4C4E-1938-46F3-8FAE-9EC8B05F0B3E}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="B3c2">Planilha1!$B$3</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -114,7 +117,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -433,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA940922-860D-4863-B9A5-E7EE2A94C235}">
-  <dimension ref="A1:G433"/>
+  <dimension ref="A1:J433"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.7109375" style="1" customWidth="1"/>
@@ -445,7 +448,7 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1">
+    <row r="1" spans="1:10" s="2" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -468,54 +471,55 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:10">
       <c r="A2" s="4"/>
       <c r="G2" s="1" t="e">
         <f>MEDIAN(C2,D2,E2,F2)*1.8</f>
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:10">
       <c r="A3" s="4"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:7">
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="4"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:10">
       <c r="A5" s="4"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:10">
       <c r="A6" s="4"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:10">
       <c r="A7" s="4"/>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" s="4"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:10">
       <c r="A9" s="4"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:10">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:10">
       <c r="A11" s="4"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:10">
       <c r="A12" s="4"/>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="4"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:10">
       <c r="A14" s="4"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:10">
       <c r="A15" s="4"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:10">
       <c r="A16" s="4"/>
     </row>
     <row r="17" spans="1:1">
@@ -1771,137 +1775,6 @@
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="A431:A433"/>
-    <mergeCell ref="A416:A418"/>
-    <mergeCell ref="A419:A421"/>
-    <mergeCell ref="A422:A424"/>
-    <mergeCell ref="A425:A427"/>
-    <mergeCell ref="A428:A430"/>
-    <mergeCell ref="A401:A403"/>
-    <mergeCell ref="A404:A406"/>
-    <mergeCell ref="A407:A409"/>
-    <mergeCell ref="A410:A412"/>
-    <mergeCell ref="A413:A415"/>
-    <mergeCell ref="A386:A388"/>
-    <mergeCell ref="A389:A391"/>
-    <mergeCell ref="A392:A394"/>
-    <mergeCell ref="A395:A397"/>
-    <mergeCell ref="A398:A400"/>
-    <mergeCell ref="A371:A373"/>
-    <mergeCell ref="A374:A376"/>
-    <mergeCell ref="A377:A379"/>
-    <mergeCell ref="A380:A382"/>
-    <mergeCell ref="A383:A385"/>
-    <mergeCell ref="A356:A358"/>
-    <mergeCell ref="A359:A361"/>
-    <mergeCell ref="A362:A364"/>
-    <mergeCell ref="A365:A367"/>
-    <mergeCell ref="A368:A370"/>
-    <mergeCell ref="A341:A343"/>
-    <mergeCell ref="A344:A346"/>
-    <mergeCell ref="A347:A349"/>
-    <mergeCell ref="A350:A352"/>
-    <mergeCell ref="A353:A355"/>
-    <mergeCell ref="A326:A328"/>
-    <mergeCell ref="A329:A331"/>
-    <mergeCell ref="A332:A334"/>
-    <mergeCell ref="A335:A337"/>
-    <mergeCell ref="A338:A340"/>
-    <mergeCell ref="A311:A313"/>
-    <mergeCell ref="A314:A316"/>
-    <mergeCell ref="A317:A319"/>
-    <mergeCell ref="A320:A322"/>
-    <mergeCell ref="A323:A325"/>
-    <mergeCell ref="A296:A298"/>
-    <mergeCell ref="A299:A301"/>
-    <mergeCell ref="A302:A304"/>
-    <mergeCell ref="A305:A307"/>
-    <mergeCell ref="A308:A310"/>
-    <mergeCell ref="A281:A283"/>
-    <mergeCell ref="A284:A286"/>
-    <mergeCell ref="A287:A289"/>
-    <mergeCell ref="A290:A292"/>
-    <mergeCell ref="A293:A295"/>
-    <mergeCell ref="A266:A268"/>
-    <mergeCell ref="A269:A271"/>
-    <mergeCell ref="A272:A274"/>
-    <mergeCell ref="A275:A277"/>
-    <mergeCell ref="A278:A280"/>
-    <mergeCell ref="A251:A253"/>
-    <mergeCell ref="A254:A256"/>
-    <mergeCell ref="A257:A259"/>
-    <mergeCell ref="A260:A262"/>
-    <mergeCell ref="A263:A265"/>
-    <mergeCell ref="A236:A238"/>
-    <mergeCell ref="A239:A241"/>
-    <mergeCell ref="A242:A244"/>
-    <mergeCell ref="A245:A247"/>
-    <mergeCell ref="A248:A250"/>
-    <mergeCell ref="A221:A223"/>
-    <mergeCell ref="A224:A226"/>
-    <mergeCell ref="A227:A229"/>
-    <mergeCell ref="A230:A232"/>
-    <mergeCell ref="A233:A235"/>
-    <mergeCell ref="A206:A208"/>
-    <mergeCell ref="A209:A211"/>
-    <mergeCell ref="A212:A214"/>
-    <mergeCell ref="A215:A217"/>
-    <mergeCell ref="A218:A220"/>
-    <mergeCell ref="A191:A193"/>
-    <mergeCell ref="A194:A196"/>
-    <mergeCell ref="A197:A199"/>
-    <mergeCell ref="A200:A202"/>
-    <mergeCell ref="A203:A205"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A181"/>
-    <mergeCell ref="A182:A184"/>
-    <mergeCell ref="A185:A187"/>
-    <mergeCell ref="A188:A190"/>
-    <mergeCell ref="A161:A163"/>
-    <mergeCell ref="A164:A166"/>
-    <mergeCell ref="A167:A169"/>
-    <mergeCell ref="A170:A172"/>
-    <mergeCell ref="A173:A175"/>
-    <mergeCell ref="A146:A148"/>
-    <mergeCell ref="A149:A151"/>
-    <mergeCell ref="A152:A154"/>
-    <mergeCell ref="A155:A157"/>
-    <mergeCell ref="A158:A160"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="A134:A136"/>
-    <mergeCell ref="A137:A139"/>
-    <mergeCell ref="A140:A142"/>
-    <mergeCell ref="A143:A145"/>
-    <mergeCell ref="A116:A118"/>
-    <mergeCell ref="A119:A121"/>
-    <mergeCell ref="A122:A124"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A112"/>
-    <mergeCell ref="A113:A115"/>
-    <mergeCell ref="A86:A88"/>
-    <mergeCell ref="A89:A91"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A98:A100"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A56:A58"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="A68:A70"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="A53:A55"/>
     <mergeCell ref="A26:A28"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="A32:A34"/>
@@ -1915,6 +1788,137 @@
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A56:A58"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="A68:A70"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="A53:A55"/>
+    <mergeCell ref="A86:A88"/>
+    <mergeCell ref="A89:A91"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="A98:A100"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A74:A76"/>
+    <mergeCell ref="A77:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A116:A118"/>
+    <mergeCell ref="A119:A121"/>
+    <mergeCell ref="A122:A124"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="A113:A115"/>
+    <mergeCell ref="A146:A148"/>
+    <mergeCell ref="A149:A151"/>
+    <mergeCell ref="A152:A154"/>
+    <mergeCell ref="A155:A157"/>
+    <mergeCell ref="A158:A160"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="A134:A136"/>
+    <mergeCell ref="A137:A139"/>
+    <mergeCell ref="A140:A142"/>
+    <mergeCell ref="A143:A145"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A181"/>
+    <mergeCell ref="A182:A184"/>
+    <mergeCell ref="A185:A187"/>
+    <mergeCell ref="A188:A190"/>
+    <mergeCell ref="A161:A163"/>
+    <mergeCell ref="A164:A166"/>
+    <mergeCell ref="A167:A169"/>
+    <mergeCell ref="A170:A172"/>
+    <mergeCell ref="A173:A175"/>
+    <mergeCell ref="A206:A208"/>
+    <mergeCell ref="A209:A211"/>
+    <mergeCell ref="A212:A214"/>
+    <mergeCell ref="A215:A217"/>
+    <mergeCell ref="A218:A220"/>
+    <mergeCell ref="A191:A193"/>
+    <mergeCell ref="A194:A196"/>
+    <mergeCell ref="A197:A199"/>
+    <mergeCell ref="A200:A202"/>
+    <mergeCell ref="A203:A205"/>
+    <mergeCell ref="A236:A238"/>
+    <mergeCell ref="A239:A241"/>
+    <mergeCell ref="A242:A244"/>
+    <mergeCell ref="A245:A247"/>
+    <mergeCell ref="A248:A250"/>
+    <mergeCell ref="A221:A223"/>
+    <mergeCell ref="A224:A226"/>
+    <mergeCell ref="A227:A229"/>
+    <mergeCell ref="A230:A232"/>
+    <mergeCell ref="A233:A235"/>
+    <mergeCell ref="A266:A268"/>
+    <mergeCell ref="A269:A271"/>
+    <mergeCell ref="A272:A274"/>
+    <mergeCell ref="A275:A277"/>
+    <mergeCell ref="A278:A280"/>
+    <mergeCell ref="A251:A253"/>
+    <mergeCell ref="A254:A256"/>
+    <mergeCell ref="A257:A259"/>
+    <mergeCell ref="A260:A262"/>
+    <mergeCell ref="A263:A265"/>
+    <mergeCell ref="A296:A298"/>
+    <mergeCell ref="A299:A301"/>
+    <mergeCell ref="A302:A304"/>
+    <mergeCell ref="A305:A307"/>
+    <mergeCell ref="A308:A310"/>
+    <mergeCell ref="A281:A283"/>
+    <mergeCell ref="A284:A286"/>
+    <mergeCell ref="A287:A289"/>
+    <mergeCell ref="A290:A292"/>
+    <mergeCell ref="A293:A295"/>
+    <mergeCell ref="A326:A328"/>
+    <mergeCell ref="A329:A331"/>
+    <mergeCell ref="A332:A334"/>
+    <mergeCell ref="A335:A337"/>
+    <mergeCell ref="A338:A340"/>
+    <mergeCell ref="A311:A313"/>
+    <mergeCell ref="A314:A316"/>
+    <mergeCell ref="A317:A319"/>
+    <mergeCell ref="A320:A322"/>
+    <mergeCell ref="A323:A325"/>
+    <mergeCell ref="A356:A358"/>
+    <mergeCell ref="A359:A361"/>
+    <mergeCell ref="A362:A364"/>
+    <mergeCell ref="A365:A367"/>
+    <mergeCell ref="A368:A370"/>
+    <mergeCell ref="A341:A343"/>
+    <mergeCell ref="A344:A346"/>
+    <mergeCell ref="A347:A349"/>
+    <mergeCell ref="A350:A352"/>
+    <mergeCell ref="A353:A355"/>
+    <mergeCell ref="A386:A388"/>
+    <mergeCell ref="A389:A391"/>
+    <mergeCell ref="A392:A394"/>
+    <mergeCell ref="A395:A397"/>
+    <mergeCell ref="A398:A400"/>
+    <mergeCell ref="A371:A373"/>
+    <mergeCell ref="A374:A376"/>
+    <mergeCell ref="A377:A379"/>
+    <mergeCell ref="A380:A382"/>
+    <mergeCell ref="A383:A385"/>
+    <mergeCell ref="A431:A433"/>
+    <mergeCell ref="A416:A418"/>
+    <mergeCell ref="A419:A421"/>
+    <mergeCell ref="A422:A424"/>
+    <mergeCell ref="A425:A427"/>
+    <mergeCell ref="A428:A430"/>
+    <mergeCell ref="A401:A403"/>
+    <mergeCell ref="A404:A406"/>
+    <mergeCell ref="A407:A409"/>
+    <mergeCell ref="A410:A412"/>
+    <mergeCell ref="A413:A415"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Migração para o outro computador e Correção do erro de 2 peças da compel
</commit_message>
<xml_diff>
--- a/planilhas/Planilha de Base para Cotacao.xlsx
+++ b/planilhas/Planilha de Base para Cotacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a19316afdd125d6/Documentos/GitHub/hawks-automations/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="390" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B32C1AE-7E22-4C86-A523-74AF08821354}"/>
+  <xr:revisionPtr revIDLastSave="419" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A015A2A-0D5F-4772-BE4A-F77452162B70}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{AB0A4C4E-1938-46F3-8FAE-9EC8B05F0B3E}"/>
   </bookViews>
@@ -447,7 +447,7 @@
   <dimension ref="A1:J433"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="45" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57" style="3" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
@@ -1781,137 +1781,6 @@
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="A431:A433"/>
-    <mergeCell ref="A416:A418"/>
-    <mergeCell ref="A419:A421"/>
-    <mergeCell ref="A422:A424"/>
-    <mergeCell ref="A425:A427"/>
-    <mergeCell ref="A428:A430"/>
-    <mergeCell ref="A401:A403"/>
-    <mergeCell ref="A404:A406"/>
-    <mergeCell ref="A407:A409"/>
-    <mergeCell ref="A410:A412"/>
-    <mergeCell ref="A413:A415"/>
-    <mergeCell ref="A386:A388"/>
-    <mergeCell ref="A389:A391"/>
-    <mergeCell ref="A392:A394"/>
-    <mergeCell ref="A395:A397"/>
-    <mergeCell ref="A398:A400"/>
-    <mergeCell ref="A371:A373"/>
-    <mergeCell ref="A374:A376"/>
-    <mergeCell ref="A377:A379"/>
-    <mergeCell ref="A380:A382"/>
-    <mergeCell ref="A383:A385"/>
-    <mergeCell ref="A356:A358"/>
-    <mergeCell ref="A359:A361"/>
-    <mergeCell ref="A362:A364"/>
-    <mergeCell ref="A365:A367"/>
-    <mergeCell ref="A368:A370"/>
-    <mergeCell ref="A341:A343"/>
-    <mergeCell ref="A344:A346"/>
-    <mergeCell ref="A347:A349"/>
-    <mergeCell ref="A350:A352"/>
-    <mergeCell ref="A353:A355"/>
-    <mergeCell ref="A326:A328"/>
-    <mergeCell ref="A329:A331"/>
-    <mergeCell ref="A332:A334"/>
-    <mergeCell ref="A335:A337"/>
-    <mergeCell ref="A338:A340"/>
-    <mergeCell ref="A311:A313"/>
-    <mergeCell ref="A314:A316"/>
-    <mergeCell ref="A317:A319"/>
-    <mergeCell ref="A320:A322"/>
-    <mergeCell ref="A323:A325"/>
-    <mergeCell ref="A296:A298"/>
-    <mergeCell ref="A299:A301"/>
-    <mergeCell ref="A302:A304"/>
-    <mergeCell ref="A305:A307"/>
-    <mergeCell ref="A308:A310"/>
-    <mergeCell ref="A281:A283"/>
-    <mergeCell ref="A284:A286"/>
-    <mergeCell ref="A287:A289"/>
-    <mergeCell ref="A290:A292"/>
-    <mergeCell ref="A293:A295"/>
-    <mergeCell ref="A266:A268"/>
-    <mergeCell ref="A269:A271"/>
-    <mergeCell ref="A272:A274"/>
-    <mergeCell ref="A275:A277"/>
-    <mergeCell ref="A278:A280"/>
-    <mergeCell ref="A251:A253"/>
-    <mergeCell ref="A254:A256"/>
-    <mergeCell ref="A257:A259"/>
-    <mergeCell ref="A260:A262"/>
-    <mergeCell ref="A263:A265"/>
-    <mergeCell ref="A236:A238"/>
-    <mergeCell ref="A239:A241"/>
-    <mergeCell ref="A242:A244"/>
-    <mergeCell ref="A245:A247"/>
-    <mergeCell ref="A248:A250"/>
-    <mergeCell ref="A221:A223"/>
-    <mergeCell ref="A224:A226"/>
-    <mergeCell ref="A227:A229"/>
-    <mergeCell ref="A230:A232"/>
-    <mergeCell ref="A233:A235"/>
-    <mergeCell ref="A206:A208"/>
-    <mergeCell ref="A209:A211"/>
-    <mergeCell ref="A212:A214"/>
-    <mergeCell ref="A215:A217"/>
-    <mergeCell ref="A218:A220"/>
-    <mergeCell ref="A191:A193"/>
-    <mergeCell ref="A194:A196"/>
-    <mergeCell ref="A197:A199"/>
-    <mergeCell ref="A200:A202"/>
-    <mergeCell ref="A203:A205"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A181"/>
-    <mergeCell ref="A182:A184"/>
-    <mergeCell ref="A185:A187"/>
-    <mergeCell ref="A188:A190"/>
-    <mergeCell ref="A161:A163"/>
-    <mergeCell ref="A164:A166"/>
-    <mergeCell ref="A167:A169"/>
-    <mergeCell ref="A170:A172"/>
-    <mergeCell ref="A173:A175"/>
-    <mergeCell ref="A146:A148"/>
-    <mergeCell ref="A149:A151"/>
-    <mergeCell ref="A152:A154"/>
-    <mergeCell ref="A155:A157"/>
-    <mergeCell ref="A158:A160"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="A134:A136"/>
-    <mergeCell ref="A137:A139"/>
-    <mergeCell ref="A140:A142"/>
-    <mergeCell ref="A143:A145"/>
-    <mergeCell ref="A116:A118"/>
-    <mergeCell ref="A119:A121"/>
-    <mergeCell ref="A122:A124"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A112"/>
-    <mergeCell ref="A113:A115"/>
-    <mergeCell ref="A86:A88"/>
-    <mergeCell ref="A89:A91"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A98:A100"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A56:A58"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="A68:A70"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="A53:A55"/>
     <mergeCell ref="A26:A28"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="A32:A34"/>
@@ -1925,6 +1794,137 @@
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A56:A58"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="A68:A70"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="A53:A55"/>
+    <mergeCell ref="A86:A88"/>
+    <mergeCell ref="A89:A91"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="A98:A100"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A74:A76"/>
+    <mergeCell ref="A77:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A116:A118"/>
+    <mergeCell ref="A119:A121"/>
+    <mergeCell ref="A122:A124"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="A113:A115"/>
+    <mergeCell ref="A146:A148"/>
+    <mergeCell ref="A149:A151"/>
+    <mergeCell ref="A152:A154"/>
+    <mergeCell ref="A155:A157"/>
+    <mergeCell ref="A158:A160"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="A134:A136"/>
+    <mergeCell ref="A137:A139"/>
+    <mergeCell ref="A140:A142"/>
+    <mergeCell ref="A143:A145"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A181"/>
+    <mergeCell ref="A182:A184"/>
+    <mergeCell ref="A185:A187"/>
+    <mergeCell ref="A188:A190"/>
+    <mergeCell ref="A161:A163"/>
+    <mergeCell ref="A164:A166"/>
+    <mergeCell ref="A167:A169"/>
+    <mergeCell ref="A170:A172"/>
+    <mergeCell ref="A173:A175"/>
+    <mergeCell ref="A206:A208"/>
+    <mergeCell ref="A209:A211"/>
+    <mergeCell ref="A212:A214"/>
+    <mergeCell ref="A215:A217"/>
+    <mergeCell ref="A218:A220"/>
+    <mergeCell ref="A191:A193"/>
+    <mergeCell ref="A194:A196"/>
+    <mergeCell ref="A197:A199"/>
+    <mergeCell ref="A200:A202"/>
+    <mergeCell ref="A203:A205"/>
+    <mergeCell ref="A236:A238"/>
+    <mergeCell ref="A239:A241"/>
+    <mergeCell ref="A242:A244"/>
+    <mergeCell ref="A245:A247"/>
+    <mergeCell ref="A248:A250"/>
+    <mergeCell ref="A221:A223"/>
+    <mergeCell ref="A224:A226"/>
+    <mergeCell ref="A227:A229"/>
+    <mergeCell ref="A230:A232"/>
+    <mergeCell ref="A233:A235"/>
+    <mergeCell ref="A266:A268"/>
+    <mergeCell ref="A269:A271"/>
+    <mergeCell ref="A272:A274"/>
+    <mergeCell ref="A275:A277"/>
+    <mergeCell ref="A278:A280"/>
+    <mergeCell ref="A251:A253"/>
+    <mergeCell ref="A254:A256"/>
+    <mergeCell ref="A257:A259"/>
+    <mergeCell ref="A260:A262"/>
+    <mergeCell ref="A263:A265"/>
+    <mergeCell ref="A296:A298"/>
+    <mergeCell ref="A299:A301"/>
+    <mergeCell ref="A302:A304"/>
+    <mergeCell ref="A305:A307"/>
+    <mergeCell ref="A308:A310"/>
+    <mergeCell ref="A281:A283"/>
+    <mergeCell ref="A284:A286"/>
+    <mergeCell ref="A287:A289"/>
+    <mergeCell ref="A290:A292"/>
+    <mergeCell ref="A293:A295"/>
+    <mergeCell ref="A326:A328"/>
+    <mergeCell ref="A329:A331"/>
+    <mergeCell ref="A332:A334"/>
+    <mergeCell ref="A335:A337"/>
+    <mergeCell ref="A338:A340"/>
+    <mergeCell ref="A311:A313"/>
+    <mergeCell ref="A314:A316"/>
+    <mergeCell ref="A317:A319"/>
+    <mergeCell ref="A320:A322"/>
+    <mergeCell ref="A323:A325"/>
+    <mergeCell ref="A356:A358"/>
+    <mergeCell ref="A359:A361"/>
+    <mergeCell ref="A362:A364"/>
+    <mergeCell ref="A365:A367"/>
+    <mergeCell ref="A368:A370"/>
+    <mergeCell ref="A341:A343"/>
+    <mergeCell ref="A344:A346"/>
+    <mergeCell ref="A347:A349"/>
+    <mergeCell ref="A350:A352"/>
+    <mergeCell ref="A353:A355"/>
+    <mergeCell ref="A386:A388"/>
+    <mergeCell ref="A389:A391"/>
+    <mergeCell ref="A392:A394"/>
+    <mergeCell ref="A395:A397"/>
+    <mergeCell ref="A398:A400"/>
+    <mergeCell ref="A371:A373"/>
+    <mergeCell ref="A374:A376"/>
+    <mergeCell ref="A377:A379"/>
+    <mergeCell ref="A380:A382"/>
+    <mergeCell ref="A383:A385"/>
+    <mergeCell ref="A431:A433"/>
+    <mergeCell ref="A416:A418"/>
+    <mergeCell ref="A419:A421"/>
+    <mergeCell ref="A422:A424"/>
+    <mergeCell ref="A425:A427"/>
+    <mergeCell ref="A428:A430"/>
+    <mergeCell ref="A401:A403"/>
+    <mergeCell ref="A404:A406"/>
+    <mergeCell ref="A407:A409"/>
+    <mergeCell ref="A410:A412"/>
+    <mergeCell ref="A413:A415"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Correção da segunda da pesquisa compel
</commit_message>
<xml_diff>
--- a/planilhas/Planilha de Base para Cotacao.xlsx
+++ b/planilhas/Planilha de Base para Cotacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a19316afdd125d6/Documentos/GitHub/hawks-automations/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="419" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A015A2A-0D5F-4772-BE4A-F77452162B70}"/>
+  <xr:revisionPtr revIDLastSave="435" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79574DE5-2498-4818-9B86-2B285351EB8E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{AB0A4C4E-1938-46F3-8FAE-9EC8B05F0B3E}"/>
   </bookViews>
@@ -145,6 +145,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -447,7 +451,7 @@
   <dimension ref="A1:J433"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="57" style="3" customWidth="1"/>
+    <col min="1" max="1" width="65.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
@@ -1781,6 +1785,137 @@
     </row>
   </sheetData>
   <mergeCells count="144">
+    <mergeCell ref="A431:A433"/>
+    <mergeCell ref="A416:A418"/>
+    <mergeCell ref="A419:A421"/>
+    <mergeCell ref="A422:A424"/>
+    <mergeCell ref="A425:A427"/>
+    <mergeCell ref="A428:A430"/>
+    <mergeCell ref="A401:A403"/>
+    <mergeCell ref="A404:A406"/>
+    <mergeCell ref="A407:A409"/>
+    <mergeCell ref="A410:A412"/>
+    <mergeCell ref="A413:A415"/>
+    <mergeCell ref="A386:A388"/>
+    <mergeCell ref="A389:A391"/>
+    <mergeCell ref="A392:A394"/>
+    <mergeCell ref="A395:A397"/>
+    <mergeCell ref="A398:A400"/>
+    <mergeCell ref="A371:A373"/>
+    <mergeCell ref="A374:A376"/>
+    <mergeCell ref="A377:A379"/>
+    <mergeCell ref="A380:A382"/>
+    <mergeCell ref="A383:A385"/>
+    <mergeCell ref="A356:A358"/>
+    <mergeCell ref="A359:A361"/>
+    <mergeCell ref="A362:A364"/>
+    <mergeCell ref="A365:A367"/>
+    <mergeCell ref="A368:A370"/>
+    <mergeCell ref="A341:A343"/>
+    <mergeCell ref="A344:A346"/>
+    <mergeCell ref="A347:A349"/>
+    <mergeCell ref="A350:A352"/>
+    <mergeCell ref="A353:A355"/>
+    <mergeCell ref="A326:A328"/>
+    <mergeCell ref="A329:A331"/>
+    <mergeCell ref="A332:A334"/>
+    <mergeCell ref="A335:A337"/>
+    <mergeCell ref="A338:A340"/>
+    <mergeCell ref="A311:A313"/>
+    <mergeCell ref="A314:A316"/>
+    <mergeCell ref="A317:A319"/>
+    <mergeCell ref="A320:A322"/>
+    <mergeCell ref="A323:A325"/>
+    <mergeCell ref="A296:A298"/>
+    <mergeCell ref="A299:A301"/>
+    <mergeCell ref="A302:A304"/>
+    <mergeCell ref="A305:A307"/>
+    <mergeCell ref="A308:A310"/>
+    <mergeCell ref="A281:A283"/>
+    <mergeCell ref="A284:A286"/>
+    <mergeCell ref="A287:A289"/>
+    <mergeCell ref="A290:A292"/>
+    <mergeCell ref="A293:A295"/>
+    <mergeCell ref="A266:A268"/>
+    <mergeCell ref="A269:A271"/>
+    <mergeCell ref="A272:A274"/>
+    <mergeCell ref="A275:A277"/>
+    <mergeCell ref="A278:A280"/>
+    <mergeCell ref="A251:A253"/>
+    <mergeCell ref="A254:A256"/>
+    <mergeCell ref="A257:A259"/>
+    <mergeCell ref="A260:A262"/>
+    <mergeCell ref="A263:A265"/>
+    <mergeCell ref="A236:A238"/>
+    <mergeCell ref="A239:A241"/>
+    <mergeCell ref="A242:A244"/>
+    <mergeCell ref="A245:A247"/>
+    <mergeCell ref="A248:A250"/>
+    <mergeCell ref="A221:A223"/>
+    <mergeCell ref="A224:A226"/>
+    <mergeCell ref="A227:A229"/>
+    <mergeCell ref="A230:A232"/>
+    <mergeCell ref="A233:A235"/>
+    <mergeCell ref="A206:A208"/>
+    <mergeCell ref="A209:A211"/>
+    <mergeCell ref="A212:A214"/>
+    <mergeCell ref="A215:A217"/>
+    <mergeCell ref="A218:A220"/>
+    <mergeCell ref="A191:A193"/>
+    <mergeCell ref="A194:A196"/>
+    <mergeCell ref="A197:A199"/>
+    <mergeCell ref="A200:A202"/>
+    <mergeCell ref="A203:A205"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A181"/>
+    <mergeCell ref="A182:A184"/>
+    <mergeCell ref="A185:A187"/>
+    <mergeCell ref="A188:A190"/>
+    <mergeCell ref="A161:A163"/>
+    <mergeCell ref="A164:A166"/>
+    <mergeCell ref="A167:A169"/>
+    <mergeCell ref="A170:A172"/>
+    <mergeCell ref="A173:A175"/>
+    <mergeCell ref="A146:A148"/>
+    <mergeCell ref="A149:A151"/>
+    <mergeCell ref="A152:A154"/>
+    <mergeCell ref="A155:A157"/>
+    <mergeCell ref="A158:A160"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="A134:A136"/>
+    <mergeCell ref="A137:A139"/>
+    <mergeCell ref="A140:A142"/>
+    <mergeCell ref="A143:A145"/>
+    <mergeCell ref="A116:A118"/>
+    <mergeCell ref="A119:A121"/>
+    <mergeCell ref="A122:A124"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="A113:A115"/>
+    <mergeCell ref="A86:A88"/>
+    <mergeCell ref="A89:A91"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="A98:A100"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A74:A76"/>
+    <mergeCell ref="A77:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A56:A58"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="A68:A70"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="A53:A55"/>
     <mergeCell ref="A26:A28"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="A32:A34"/>
@@ -1794,137 +1929,6 @@
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A56:A58"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="A68:A70"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="A53:A55"/>
-    <mergeCell ref="A86:A88"/>
-    <mergeCell ref="A89:A91"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A98:A100"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A116:A118"/>
-    <mergeCell ref="A119:A121"/>
-    <mergeCell ref="A122:A124"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A112"/>
-    <mergeCell ref="A113:A115"/>
-    <mergeCell ref="A146:A148"/>
-    <mergeCell ref="A149:A151"/>
-    <mergeCell ref="A152:A154"/>
-    <mergeCell ref="A155:A157"/>
-    <mergeCell ref="A158:A160"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="A134:A136"/>
-    <mergeCell ref="A137:A139"/>
-    <mergeCell ref="A140:A142"/>
-    <mergeCell ref="A143:A145"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A181"/>
-    <mergeCell ref="A182:A184"/>
-    <mergeCell ref="A185:A187"/>
-    <mergeCell ref="A188:A190"/>
-    <mergeCell ref="A161:A163"/>
-    <mergeCell ref="A164:A166"/>
-    <mergeCell ref="A167:A169"/>
-    <mergeCell ref="A170:A172"/>
-    <mergeCell ref="A173:A175"/>
-    <mergeCell ref="A206:A208"/>
-    <mergeCell ref="A209:A211"/>
-    <mergeCell ref="A212:A214"/>
-    <mergeCell ref="A215:A217"/>
-    <mergeCell ref="A218:A220"/>
-    <mergeCell ref="A191:A193"/>
-    <mergeCell ref="A194:A196"/>
-    <mergeCell ref="A197:A199"/>
-    <mergeCell ref="A200:A202"/>
-    <mergeCell ref="A203:A205"/>
-    <mergeCell ref="A236:A238"/>
-    <mergeCell ref="A239:A241"/>
-    <mergeCell ref="A242:A244"/>
-    <mergeCell ref="A245:A247"/>
-    <mergeCell ref="A248:A250"/>
-    <mergeCell ref="A221:A223"/>
-    <mergeCell ref="A224:A226"/>
-    <mergeCell ref="A227:A229"/>
-    <mergeCell ref="A230:A232"/>
-    <mergeCell ref="A233:A235"/>
-    <mergeCell ref="A266:A268"/>
-    <mergeCell ref="A269:A271"/>
-    <mergeCell ref="A272:A274"/>
-    <mergeCell ref="A275:A277"/>
-    <mergeCell ref="A278:A280"/>
-    <mergeCell ref="A251:A253"/>
-    <mergeCell ref="A254:A256"/>
-    <mergeCell ref="A257:A259"/>
-    <mergeCell ref="A260:A262"/>
-    <mergeCell ref="A263:A265"/>
-    <mergeCell ref="A296:A298"/>
-    <mergeCell ref="A299:A301"/>
-    <mergeCell ref="A302:A304"/>
-    <mergeCell ref="A305:A307"/>
-    <mergeCell ref="A308:A310"/>
-    <mergeCell ref="A281:A283"/>
-    <mergeCell ref="A284:A286"/>
-    <mergeCell ref="A287:A289"/>
-    <mergeCell ref="A290:A292"/>
-    <mergeCell ref="A293:A295"/>
-    <mergeCell ref="A326:A328"/>
-    <mergeCell ref="A329:A331"/>
-    <mergeCell ref="A332:A334"/>
-    <mergeCell ref="A335:A337"/>
-    <mergeCell ref="A338:A340"/>
-    <mergeCell ref="A311:A313"/>
-    <mergeCell ref="A314:A316"/>
-    <mergeCell ref="A317:A319"/>
-    <mergeCell ref="A320:A322"/>
-    <mergeCell ref="A323:A325"/>
-    <mergeCell ref="A356:A358"/>
-    <mergeCell ref="A359:A361"/>
-    <mergeCell ref="A362:A364"/>
-    <mergeCell ref="A365:A367"/>
-    <mergeCell ref="A368:A370"/>
-    <mergeCell ref="A341:A343"/>
-    <mergeCell ref="A344:A346"/>
-    <mergeCell ref="A347:A349"/>
-    <mergeCell ref="A350:A352"/>
-    <mergeCell ref="A353:A355"/>
-    <mergeCell ref="A386:A388"/>
-    <mergeCell ref="A389:A391"/>
-    <mergeCell ref="A392:A394"/>
-    <mergeCell ref="A395:A397"/>
-    <mergeCell ref="A398:A400"/>
-    <mergeCell ref="A371:A373"/>
-    <mergeCell ref="A374:A376"/>
-    <mergeCell ref="A377:A379"/>
-    <mergeCell ref="A380:A382"/>
-    <mergeCell ref="A383:A385"/>
-    <mergeCell ref="A431:A433"/>
-    <mergeCell ref="A416:A418"/>
-    <mergeCell ref="A419:A421"/>
-    <mergeCell ref="A422:A424"/>
-    <mergeCell ref="A425:A427"/>
-    <mergeCell ref="A428:A430"/>
-    <mergeCell ref="A401:A403"/>
-    <mergeCell ref="A404:A406"/>
-    <mergeCell ref="A407:A409"/>
-    <mergeCell ref="A410:A412"/>
-    <mergeCell ref="A413:A415"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
partial commit (rmp process)
</commit_message>
<xml_diff>
--- a/planilhas/Planilha de Base para Cotacao.xlsx
+++ b/planilhas/Planilha de Base para Cotacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a19316afdd125d6/Documentos/GitHub/hawks-automations/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="669" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D5FCF2D-A3D6-4171-992B-D2F3DF5FB523}"/>
+  <xr:revisionPtr revIDLastSave="670" documentId="8_{B6B05E56-6ADC-4554-A921-81DFAB966C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C10EC37B-2BDA-4D1C-A6BF-BDEF01CE98EB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{AB0A4C4E-1938-46F3-8FAE-9EC8B05F0B3E}"/>
   </bookViews>
@@ -38,30 +38,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Peça</t>
   </si>
@@ -85,33 +63,6 @@
   </si>
   <si>
     <t>Rmp (40)</t>
-  </si>
-  <si>
-    <t>LFR6B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VELA DE IGNIÇÃO BOSCH </t>
-  </si>
-  <si>
-    <t>Indisponível</t>
-  </si>
-  <si>
-    <t>F000KE0P31</t>
-  </si>
-  <si>
-    <t>OX3392D</t>
-  </si>
-  <si>
-    <t>HU71151X</t>
-  </si>
-  <si>
-    <t>WOE710</t>
-  </si>
-  <si>
-    <t>LX1745</t>
-  </si>
-  <si>
-    <t>C42922</t>
   </si>
 </sst>
 </file>
@@ -530,49 +481,10 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2">
-        <f>36.5 +15</f>
-        <v>51.5</v>
-      </c>
-      <c r="D2" s="2" t="e" cm="1">
-        <f t="array" ref="D2">F000KE0P51+7</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="E2" s="2">
-        <f>29.09+10</f>
-        <v>39.090000000000003</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="A2" s="5"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2">
-        <f>36.5 +15</f>
-        <v>51.5</v>
-      </c>
-      <c r="D3" s="2">
-        <f>155.34+7</f>
-        <v>162.34</v>
-      </c>
-      <c r="E3" s="2">
-        <f>33.29+10</f>
-        <v>43.29</v>
-      </c>
-      <c r="F3" s="2">
-        <f>30.42+10</f>
-        <v>40.42</v>
-      </c>
       <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -581,108 +493,19 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2">
-        <f>41.3+7</f>
-        <v>48.3</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
-      <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2">
-        <f>21.2+15</f>
-        <v>36.200000000000003</v>
-      </c>
-      <c r="D6" s="2">
-        <f>19.69+7</f>
-        <v>26.69</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="2">
-        <f>19.08+10</f>
-        <v>29.08</v>
-      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="2">
-        <f>16.7+15</f>
-        <v>31.7</v>
-      </c>
-      <c r="D7" s="2">
-        <f>15.52+7</f>
-        <v>22.52</v>
-      </c>
-      <c r="E7" s="2">
-        <f>16.47+10</f>
-        <v>26.47</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="I7" s="4"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="2">
-        <f>47.3+15</f>
-        <v>62.3</v>
-      </c>
-      <c r="D8" s="2">
-        <f>42.87+7</f>
-        <v>49.87</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="2">
-        <f>43.23+10</f>
-        <v>53.23</v>
-      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
-      <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="2">
-        <f>43.6+15</f>
-        <v>58.6</v>
-      </c>
-      <c r="D9" s="2">
-        <f>60.37+7</f>
-        <v>67.37</v>
-      </c>
-      <c r="E9" s="2">
-        <f>51.75+10</f>
-        <v>61.75</v>
-      </c>
-      <c r="F9" s="2">
-        <f>51.58+10</f>
-        <v>61.58</v>
-      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
@@ -1958,6 +1781,137 @@
     </row>
   </sheetData>
   <mergeCells count="144">
+    <mergeCell ref="A431:A433"/>
+    <mergeCell ref="A416:A418"/>
+    <mergeCell ref="A419:A421"/>
+    <mergeCell ref="A422:A424"/>
+    <mergeCell ref="A425:A427"/>
+    <mergeCell ref="A428:A430"/>
+    <mergeCell ref="A401:A403"/>
+    <mergeCell ref="A404:A406"/>
+    <mergeCell ref="A407:A409"/>
+    <mergeCell ref="A410:A412"/>
+    <mergeCell ref="A413:A415"/>
+    <mergeCell ref="A386:A388"/>
+    <mergeCell ref="A389:A391"/>
+    <mergeCell ref="A392:A394"/>
+    <mergeCell ref="A395:A397"/>
+    <mergeCell ref="A398:A400"/>
+    <mergeCell ref="A371:A373"/>
+    <mergeCell ref="A374:A376"/>
+    <mergeCell ref="A377:A379"/>
+    <mergeCell ref="A380:A382"/>
+    <mergeCell ref="A383:A385"/>
+    <mergeCell ref="A356:A358"/>
+    <mergeCell ref="A359:A361"/>
+    <mergeCell ref="A362:A364"/>
+    <mergeCell ref="A365:A367"/>
+    <mergeCell ref="A368:A370"/>
+    <mergeCell ref="A341:A343"/>
+    <mergeCell ref="A344:A346"/>
+    <mergeCell ref="A347:A349"/>
+    <mergeCell ref="A350:A352"/>
+    <mergeCell ref="A353:A355"/>
+    <mergeCell ref="A326:A328"/>
+    <mergeCell ref="A329:A331"/>
+    <mergeCell ref="A332:A334"/>
+    <mergeCell ref="A335:A337"/>
+    <mergeCell ref="A338:A340"/>
+    <mergeCell ref="A311:A313"/>
+    <mergeCell ref="A314:A316"/>
+    <mergeCell ref="A317:A319"/>
+    <mergeCell ref="A320:A322"/>
+    <mergeCell ref="A323:A325"/>
+    <mergeCell ref="A296:A298"/>
+    <mergeCell ref="A299:A301"/>
+    <mergeCell ref="A302:A304"/>
+    <mergeCell ref="A305:A307"/>
+    <mergeCell ref="A308:A310"/>
+    <mergeCell ref="A281:A283"/>
+    <mergeCell ref="A284:A286"/>
+    <mergeCell ref="A287:A289"/>
+    <mergeCell ref="A290:A292"/>
+    <mergeCell ref="A293:A295"/>
+    <mergeCell ref="A266:A268"/>
+    <mergeCell ref="A269:A271"/>
+    <mergeCell ref="A272:A274"/>
+    <mergeCell ref="A275:A277"/>
+    <mergeCell ref="A278:A280"/>
+    <mergeCell ref="A251:A253"/>
+    <mergeCell ref="A254:A256"/>
+    <mergeCell ref="A257:A259"/>
+    <mergeCell ref="A260:A262"/>
+    <mergeCell ref="A263:A265"/>
+    <mergeCell ref="A236:A238"/>
+    <mergeCell ref="A239:A241"/>
+    <mergeCell ref="A242:A244"/>
+    <mergeCell ref="A245:A247"/>
+    <mergeCell ref="A248:A250"/>
+    <mergeCell ref="A221:A223"/>
+    <mergeCell ref="A224:A226"/>
+    <mergeCell ref="A227:A229"/>
+    <mergeCell ref="A230:A232"/>
+    <mergeCell ref="A233:A235"/>
+    <mergeCell ref="A206:A208"/>
+    <mergeCell ref="A209:A211"/>
+    <mergeCell ref="A212:A214"/>
+    <mergeCell ref="A215:A217"/>
+    <mergeCell ref="A218:A220"/>
+    <mergeCell ref="A191:A193"/>
+    <mergeCell ref="A194:A196"/>
+    <mergeCell ref="A197:A199"/>
+    <mergeCell ref="A200:A202"/>
+    <mergeCell ref="A203:A205"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A181"/>
+    <mergeCell ref="A182:A184"/>
+    <mergeCell ref="A185:A187"/>
+    <mergeCell ref="A188:A190"/>
+    <mergeCell ref="A161:A163"/>
+    <mergeCell ref="A164:A166"/>
+    <mergeCell ref="A167:A169"/>
+    <mergeCell ref="A170:A172"/>
+    <mergeCell ref="A173:A175"/>
+    <mergeCell ref="A146:A148"/>
+    <mergeCell ref="A149:A151"/>
+    <mergeCell ref="A152:A154"/>
+    <mergeCell ref="A155:A157"/>
+    <mergeCell ref="A158:A160"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="A134:A136"/>
+    <mergeCell ref="A137:A139"/>
+    <mergeCell ref="A140:A142"/>
+    <mergeCell ref="A143:A145"/>
+    <mergeCell ref="A116:A118"/>
+    <mergeCell ref="A119:A121"/>
+    <mergeCell ref="A122:A124"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="A113:A115"/>
+    <mergeCell ref="A86:A88"/>
+    <mergeCell ref="A89:A91"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="A98:A100"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A74:A76"/>
+    <mergeCell ref="A77:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A56:A58"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="A68:A70"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="A53:A55"/>
     <mergeCell ref="A26:A28"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="A32:A34"/>
@@ -1971,137 +1925,6 @@
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A56:A58"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="A68:A70"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="A53:A55"/>
-    <mergeCell ref="A86:A88"/>
-    <mergeCell ref="A89:A91"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A98:A100"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A116:A118"/>
-    <mergeCell ref="A119:A121"/>
-    <mergeCell ref="A122:A124"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A112"/>
-    <mergeCell ref="A113:A115"/>
-    <mergeCell ref="A146:A148"/>
-    <mergeCell ref="A149:A151"/>
-    <mergeCell ref="A152:A154"/>
-    <mergeCell ref="A155:A157"/>
-    <mergeCell ref="A158:A160"/>
-    <mergeCell ref="A131:A133"/>
-    <mergeCell ref="A134:A136"/>
-    <mergeCell ref="A137:A139"/>
-    <mergeCell ref="A140:A142"/>
-    <mergeCell ref="A143:A145"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A181"/>
-    <mergeCell ref="A182:A184"/>
-    <mergeCell ref="A185:A187"/>
-    <mergeCell ref="A188:A190"/>
-    <mergeCell ref="A161:A163"/>
-    <mergeCell ref="A164:A166"/>
-    <mergeCell ref="A167:A169"/>
-    <mergeCell ref="A170:A172"/>
-    <mergeCell ref="A173:A175"/>
-    <mergeCell ref="A206:A208"/>
-    <mergeCell ref="A209:A211"/>
-    <mergeCell ref="A212:A214"/>
-    <mergeCell ref="A215:A217"/>
-    <mergeCell ref="A218:A220"/>
-    <mergeCell ref="A191:A193"/>
-    <mergeCell ref="A194:A196"/>
-    <mergeCell ref="A197:A199"/>
-    <mergeCell ref="A200:A202"/>
-    <mergeCell ref="A203:A205"/>
-    <mergeCell ref="A236:A238"/>
-    <mergeCell ref="A239:A241"/>
-    <mergeCell ref="A242:A244"/>
-    <mergeCell ref="A245:A247"/>
-    <mergeCell ref="A248:A250"/>
-    <mergeCell ref="A221:A223"/>
-    <mergeCell ref="A224:A226"/>
-    <mergeCell ref="A227:A229"/>
-    <mergeCell ref="A230:A232"/>
-    <mergeCell ref="A233:A235"/>
-    <mergeCell ref="A266:A268"/>
-    <mergeCell ref="A269:A271"/>
-    <mergeCell ref="A272:A274"/>
-    <mergeCell ref="A275:A277"/>
-    <mergeCell ref="A278:A280"/>
-    <mergeCell ref="A251:A253"/>
-    <mergeCell ref="A254:A256"/>
-    <mergeCell ref="A257:A259"/>
-    <mergeCell ref="A260:A262"/>
-    <mergeCell ref="A263:A265"/>
-    <mergeCell ref="A296:A298"/>
-    <mergeCell ref="A299:A301"/>
-    <mergeCell ref="A302:A304"/>
-    <mergeCell ref="A305:A307"/>
-    <mergeCell ref="A308:A310"/>
-    <mergeCell ref="A281:A283"/>
-    <mergeCell ref="A284:A286"/>
-    <mergeCell ref="A287:A289"/>
-    <mergeCell ref="A290:A292"/>
-    <mergeCell ref="A293:A295"/>
-    <mergeCell ref="A326:A328"/>
-    <mergeCell ref="A329:A331"/>
-    <mergeCell ref="A332:A334"/>
-    <mergeCell ref="A335:A337"/>
-    <mergeCell ref="A338:A340"/>
-    <mergeCell ref="A311:A313"/>
-    <mergeCell ref="A314:A316"/>
-    <mergeCell ref="A317:A319"/>
-    <mergeCell ref="A320:A322"/>
-    <mergeCell ref="A323:A325"/>
-    <mergeCell ref="A356:A358"/>
-    <mergeCell ref="A359:A361"/>
-    <mergeCell ref="A362:A364"/>
-    <mergeCell ref="A365:A367"/>
-    <mergeCell ref="A368:A370"/>
-    <mergeCell ref="A341:A343"/>
-    <mergeCell ref="A344:A346"/>
-    <mergeCell ref="A347:A349"/>
-    <mergeCell ref="A350:A352"/>
-    <mergeCell ref="A353:A355"/>
-    <mergeCell ref="A386:A388"/>
-    <mergeCell ref="A389:A391"/>
-    <mergeCell ref="A392:A394"/>
-    <mergeCell ref="A395:A397"/>
-    <mergeCell ref="A398:A400"/>
-    <mergeCell ref="A371:A373"/>
-    <mergeCell ref="A374:A376"/>
-    <mergeCell ref="A377:A379"/>
-    <mergeCell ref="A380:A382"/>
-    <mergeCell ref="A383:A385"/>
-    <mergeCell ref="A431:A433"/>
-    <mergeCell ref="A416:A418"/>
-    <mergeCell ref="A419:A421"/>
-    <mergeCell ref="A422:A424"/>
-    <mergeCell ref="A425:A427"/>
-    <mergeCell ref="A428:A430"/>
-    <mergeCell ref="A401:A403"/>
-    <mergeCell ref="A404:A406"/>
-    <mergeCell ref="A407:A409"/>
-    <mergeCell ref="A410:A412"/>
-    <mergeCell ref="A413:A415"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>